<commit_message>
White out-of-month areas on the ACS 2027 calendar
The grey blocks outside each month's span are cleared to plain white,
so only real days carry the grid and weekend shading.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLo1WfwUDkbwfJEF3ZNVbB
</commit_message>
<xml_diff>
--- a/output/acs-activity-calendar-2027.xlsx
+++ b/output/acs-activity-calendar-2027.xlsx
@@ -2574,7 +2574,7 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1283">
+  <cellXfs count="1287">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -6459,6 +6459,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="109" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="149" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="149" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="149" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="149" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -7433,7 +7445,7 @@
           <t>January</t>
         </is>
       </c>
-      <c r="B4" s="1266" t="n"/>
+      <c r="B4" s="1283" t="n"/>
       <c r="F4" s="1149" t="n"/>
       <c r="G4" s="1238" t="n">
         <v>1</v>
@@ -7528,7 +7540,7 @@
       <c r="AK4" s="1239" t="n">
         <v>31</v>
       </c>
-      <c r="AL4" s="1267" t="n"/>
+      <c r="AL4" s="1284" t="n"/>
       <c r="AN4" s="1149" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -8081,7 +8093,7 @@
           <t>February</t>
         </is>
       </c>
-      <c r="B18" s="1277" t="n"/>
+      <c r="B18" s="1285" t="n"/>
       <c r="I18" s="1149" t="n"/>
       <c r="J18" s="1238" t="n">
         <v>1</v>
@@ -8167,7 +8179,7 @@
       <c r="AK18" s="1239" t="n">
         <v>28</v>
       </c>
-      <c r="AL18" s="1278" t="n"/>
+      <c r="AL18" s="1286" t="n"/>
       <c r="AN18" s="1149" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" thickBot="1">
@@ -8695,7 +8707,7 @@
           <t>March</t>
         </is>
       </c>
-      <c r="B32" s="1278" t="n"/>
+      <c r="B32" s="1286" t="n"/>
       <c r="I32" s="1149" t="n"/>
       <c r="J32" s="1238" t="n">
         <v>1</v>
@@ -9311,7 +9323,7 @@
           <t>April</t>
         </is>
       </c>
-      <c r="B45" s="1278" t="n"/>
+      <c r="B45" s="1286" t="n"/>
       <c r="E45" s="1149" t="n"/>
       <c r="F45" s="1238" t="n">
         <v>1</v>
@@ -9403,7 +9415,7 @@
       <c r="AI45" s="1238" t="n">
         <v>30</v>
       </c>
-      <c r="AJ45" s="1266" t="n"/>
+      <c r="AJ45" s="1283" t="n"/>
       <c r="AN45" s="1149" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1">
@@ -9906,7 +9918,7 @@
           <t>May</t>
         </is>
       </c>
-      <c r="B58" s="1278" t="n"/>
+      <c r="B58" s="1286" t="n"/>
       <c r="G58" s="1149" t="n"/>
       <c r="H58" s="1239" t="n">
         <v>1</v>
@@ -10001,7 +10013,7 @@
       <c r="AL58" s="1238" t="n">
         <v>31</v>
       </c>
-      <c r="AM58" s="1278" t="n"/>
+      <c r="AM58" s="1286" t="n"/>
       <c r="AN58" s="1149" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" thickBot="1">
@@ -10522,7 +10534,7 @@
           <t>June</t>
         </is>
       </c>
-      <c r="B71" s="1266" t="n"/>
+      <c r="B71" s="1283" t="n"/>
       <c r="C71" s="1149" t="n"/>
       <c r="D71" s="1238" t="n">
         <v>1</v>
@@ -10614,7 +10626,7 @@
       <c r="AG71" s="1238" t="n">
         <v>30</v>
       </c>
-      <c r="AH71" s="1266" t="n"/>
+      <c r="AH71" s="1283" t="n"/>
       <c r="AN71" s="1149" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" thickBot="1">
@@ -11121,7 +11133,7 @@
           <t>July</t>
         </is>
       </c>
-      <c r="B84" s="1278" t="n"/>
+      <c r="B84" s="1286" t="n"/>
       <c r="E84" s="1149" t="n"/>
       <c r="F84" s="1238" t="n">
         <v>1</v>
@@ -11216,7 +11228,7 @@
       <c r="AJ84" s="1239" t="n">
         <v>31</v>
       </c>
-      <c r="AK84" s="1266" t="n"/>
+      <c r="AK84" s="1283" t="n"/>
       <c r="AN84" s="1149" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" thickBot="1">
@@ -11725,7 +11737,7 @@
           <t>August</t>
         </is>
       </c>
-      <c r="B97" s="1278" t="n"/>
+      <c r="B97" s="1286" t="n"/>
       <c r="H97" s="1149" t="n"/>
       <c r="I97" s="1239" t="n">
         <v>1</v>
@@ -11820,7 +11832,7 @@
       <c r="AM97" s="1238" t="n">
         <v>31</v>
       </c>
-      <c r="AN97" s="1266" t="n"/>
+      <c r="AN97" s="1283" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="1241" t="inlineStr">
@@ -12368,7 +12380,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="B111" s="1278" t="n"/>
+      <c r="B111" s="1286" t="n"/>
       <c r="D111" s="1149" t="n"/>
       <c r="E111" s="1238" t="n">
         <v>1</v>
@@ -12460,7 +12472,7 @@
       <c r="AH111" s="1238" t="n">
         <v>30</v>
       </c>
-      <c r="AI111" s="1266" t="n"/>
+      <c r="AI111" s="1283" t="n"/>
       <c r="AN111" s="1149" t="n"/>
     </row>
     <row r="112" ht="15" customHeight="1">
@@ -12975,7 +12987,7 @@
           <t>October</t>
         </is>
       </c>
-      <c r="B124" s="1266" t="n"/>
+      <c r="B124" s="1283" t="n"/>
       <c r="F124" s="1149" t="n"/>
       <c r="G124" s="1238" t="n">
         <v>1</v>
@@ -13070,7 +13082,7 @@
       <c r="AK124" s="1239" t="n">
         <v>31</v>
       </c>
-      <c r="AL124" s="1278" t="n"/>
+      <c r="AL124" s="1286" t="n"/>
       <c r="AN124" s="1149" t="n"/>
     </row>
     <row r="125" ht="15" customHeight="1">
@@ -13583,7 +13595,7 @@
           <t>November</t>
         </is>
       </c>
-      <c r="B137" s="1278" t="n"/>
+      <c r="B137" s="1286" t="n"/>
       <c r="I137" s="1149" t="n"/>
       <c r="J137" s="1238" t="n">
         <v>1</v>
@@ -13675,7 +13687,7 @@
       <c r="AM137" s="1238" t="n">
         <v>30</v>
       </c>
-      <c r="AN137" s="1278" t="n"/>
+      <c r="AN137" s="1286" t="n"/>
     </row>
     <row r="138" ht="15" customHeight="1" thickBot="1">
       <c r="A138" s="1241" t="inlineStr">
@@ -14181,7 +14193,7 @@
           <t>December</t>
         </is>
       </c>
-      <c r="B150" s="1266" t="n"/>
+      <c r="B150" s="1283" t="n"/>
       <c r="D150" s="1149" t="n"/>
       <c r="E150" s="1238" t="n">
         <v>1</v>
@@ -14276,7 +14288,7 @@
       <c r="AI150" s="1238" t="n">
         <v>31</v>
       </c>
-      <c r="AJ150" s="1266" t="n"/>
+      <c r="AJ150" s="1283" t="n"/>
       <c r="AN150" s="1149" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1" thickBot="1">
@@ -15068,8 +15080,8 @@
     <mergeCell ref="D81:U81"/>
     <mergeCell ref="P131:U131"/>
     <mergeCell ref="J42:W42"/>
+    <mergeCell ref="J147:AB147"/>
     <mergeCell ref="G131:H131"/>
-    <mergeCell ref="J147:AB147"/>
     <mergeCell ref="AN97:AN109"/>
     <mergeCell ref="V41:AB41"/>
     <mergeCell ref="AE13:AK13"/>

</xml_diff>

<commit_message>
Align ALC activities to their wing rows with LD/ELDA prefixes
Misplaced bars are moved to the correct lanes: February's LD courses
off the OCS row and its ELDA courses off the LD row, and March's wing
activities off the ACS rows. Every LD Wing bar now starts with LD and
every ELDA bar with ELDA. Vacated cells return to plain grid styling.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLo1WfwUDkbwfJEF3ZNVbB
</commit_message>
<xml_diff>
--- a/output/acs-activity-calendar-2027.xlsx
+++ b/output/acs-activity-calendar-2027.xlsx
@@ -828,7 +828,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="153">
+  <borders count="155">
     <border>
       <left/>
       <right/>
@@ -2554,6 +2554,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color rgb="00C8C6BD"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="00C8C6BD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color rgb="00C8C6BD"/>
+      </right>
+      <top style="hair">
+        <color rgb="00C8C6BD"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="00C8C6BD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2574,7 +2598,7 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1287">
+  <cellXfs count="1294">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -6472,6 +6496,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="149" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="103" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="53" borderId="146" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="53" borderId="146" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="51" borderId="103" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="54" borderId="146" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="54" borderId="146" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="53" borderId="146" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7789,7 +7832,7 @@
       <c r="K11" s="1013" t="n"/>
       <c r="L11" s="1273" t="inlineStr">
         <is>
-          <t>TtT TFCC</t>
+          <t>LD TtT TFCC</t>
         </is>
       </c>
       <c r="M11" s="1155" t="n"/>
@@ -7805,7 +7848,7 @@
       <c r="W11" s="1012" t="n"/>
       <c r="X11" s="1273" t="inlineStr">
         <is>
-          <t>LEAD TEAMS BMC</t>
+          <t>LD LEAD TEAMS BMC</t>
         </is>
       </c>
       <c r="Y11" s="1155" t="n"/>
@@ -7842,7 +7885,7 @@
       <c r="P12" s="1012" t="n"/>
       <c r="Q12" s="1274" t="inlineStr">
         <is>
-          <t>LEAD TEAMS BMC</t>
+          <t>ELDA LEAD TEAMS BMC</t>
         </is>
       </c>
       <c r="R12" s="1155" t="n"/>
@@ -7860,7 +7903,7 @@
       <c r="AD12" s="1012" t="n"/>
       <c r="AE12" s="1274" t="inlineStr">
         <is>
-          <t>LEAD TEAMS LMC</t>
+          <t>ELDA LEAD TEAMS LMC</t>
         </is>
       </c>
       <c r="AF12" s="1155" t="n"/>
@@ -8370,15 +8413,11 @@
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="1268" t="n"/>
       <c r="I24" s="1149" t="n"/>
-      <c r="J24" s="1273" t="inlineStr">
-        <is>
-          <t>LEAD TEAMS LMC</t>
-        </is>
-      </c>
-      <c r="K24" s="1155" t="n"/>
-      <c r="L24" s="1155" t="n"/>
-      <c r="M24" s="1155" t="n"/>
-      <c r="N24" s="1156" t="n"/>
+      <c r="J24" s="1287" t="n"/>
+      <c r="K24" s="1003" t="n"/>
+      <c r="L24" s="1003" t="n"/>
+      <c r="M24" s="1003" t="n"/>
+      <c r="N24" s="1003" t="n"/>
       <c r="O24" s="1015" t="n"/>
       <c r="P24" s="1015" t="n"/>
       <c r="Q24" s="1043" t="n"/>
@@ -8388,15 +8427,11 @@
       <c r="U24" s="1024" t="n"/>
       <c r="V24" s="1012" t="n"/>
       <c r="W24" s="1012" t="n"/>
-      <c r="X24" s="1273" t="inlineStr">
-        <is>
-          <t>LEAD LEADERS BMC</t>
-        </is>
-      </c>
-      <c r="Y24" s="1155" t="n"/>
-      <c r="Z24" s="1155" t="n"/>
-      <c r="AA24" s="1155" t="n"/>
-      <c r="AB24" s="1156" t="n"/>
+      <c r="X24" s="1287" t="n"/>
+      <c r="Y24" s="1003" t="n"/>
+      <c r="Z24" s="1003" t="n"/>
+      <c r="AA24" s="1003" t="n"/>
+      <c r="AB24" s="1003" t="n"/>
       <c r="AC24" s="1012" t="n"/>
       <c r="AD24" s="1012" t="n"/>
       <c r="AE24" s="1024" t="n"/>
@@ -8415,41 +8450,41 @@
         </is>
       </c>
       <c r="I25" s="1149" t="n"/>
-      <c r="J25" s="1024" t="n"/>
-      <c r="K25" s="1024" t="n"/>
-      <c r="L25" s="1024" t="n"/>
-      <c r="M25" s="1024" t="n"/>
-      <c r="N25" s="1008" t="n"/>
+      <c r="J25" s="1288" t="inlineStr">
+        <is>
+          <t>LD LEAD TEAMS LMC</t>
+        </is>
+      </c>
+      <c r="K25" s="1289" t="n"/>
+      <c r="L25" s="1289" t="n"/>
+      <c r="M25" s="1289" t="n"/>
+      <c r="N25" s="1289" t="n"/>
       <c r="O25" s="1012" t="n"/>
       <c r="P25" s="1012" t="n"/>
-      <c r="Q25" s="1274" t="inlineStr">
-        <is>
-          <t>LEAD LEADERS BMC</t>
-        </is>
-      </c>
-      <c r="R25" s="1155" t="n"/>
-      <c r="S25" s="1155" t="n"/>
-      <c r="T25" s="1155" t="n"/>
-      <c r="U25" s="1155" t="n"/>
-      <c r="V25" s="1156" t="n"/>
+      <c r="Q25" s="1287" t="n"/>
+      <c r="R25" s="1003" t="n"/>
+      <c r="S25" s="1003" t="n"/>
+      <c r="T25" s="1003" t="n"/>
+      <c r="U25" s="1003" t="n"/>
+      <c r="V25" s="1290" t="n"/>
       <c r="W25" s="1012" t="n"/>
-      <c r="X25" s="1024" t="n"/>
-      <c r="Y25" s="1024" t="n"/>
-      <c r="Z25" s="1024" t="n"/>
-      <c r="AA25" s="1024" t="n"/>
-      <c r="AB25" s="1024" t="n"/>
+      <c r="X25" s="1288" t="inlineStr">
+        <is>
+          <t>LD LEAD LEADERS BMC</t>
+        </is>
+      </c>
+      <c r="Y25" s="1289" t="n"/>
+      <c r="Z25" s="1289" t="n"/>
+      <c r="AA25" s="1289" t="n"/>
+      <c r="AB25" s="1289" t="n"/>
       <c r="AC25" s="1012" t="n"/>
       <c r="AD25" s="1012" t="n"/>
-      <c r="AE25" s="1274" t="inlineStr">
-        <is>
-          <t>LEAD LEADERS OFFICER</t>
-        </is>
-      </c>
-      <c r="AF25" s="1155" t="n"/>
-      <c r="AG25" s="1155" t="n"/>
-      <c r="AH25" s="1155" t="n"/>
-      <c r="AI25" s="1155" t="n"/>
-      <c r="AJ25" s="1156" t="n"/>
+      <c r="AE25" s="1287" t="n"/>
+      <c r="AF25" s="1003" t="n"/>
+      <c r="AG25" s="1003" t="n"/>
+      <c r="AH25" s="1003" t="n"/>
+      <c r="AI25" s="1003" t="n"/>
+      <c r="AJ25" s="1290" t="n"/>
       <c r="AK25" s="1045" t="n"/>
       <c r="AN25" s="1149" t="n"/>
     </row>
@@ -8467,12 +8502,16 @@
       <c r="N26" s="1008" t="n"/>
       <c r="O26" s="1012" t="n"/>
       <c r="P26" s="1012" t="n"/>
-      <c r="Q26" s="1043" t="n"/>
-      <c r="R26" s="1024" t="n"/>
-      <c r="S26" s="1024" t="n"/>
-      <c r="T26" s="1024" t="n"/>
-      <c r="U26" s="1024" t="n"/>
-      <c r="V26" s="1012" t="n"/>
+      <c r="Q26" s="1291" t="inlineStr">
+        <is>
+          <t>ELDA LEAD LEADERS BMC</t>
+        </is>
+      </c>
+      <c r="R26" s="1292" t="n"/>
+      <c r="S26" s="1292" t="n"/>
+      <c r="T26" s="1292" t="n"/>
+      <c r="U26" s="1292" t="n"/>
+      <c r="V26" s="1292" t="n"/>
       <c r="W26" s="1012" t="n"/>
       <c r="X26" s="1024" t="n"/>
       <c r="Y26" s="1024" t="n"/>
@@ -8481,12 +8520,16 @@
       <c r="AB26" s="1024" t="n"/>
       <c r="AC26" s="1043" t="n"/>
       <c r="AD26" s="1012" t="n"/>
-      <c r="AE26" s="1024" t="n"/>
-      <c r="AF26" s="1024" t="n"/>
-      <c r="AG26" s="1024" t="n"/>
-      <c r="AH26" s="1024" t="n"/>
-      <c r="AI26" s="1024" t="n"/>
-      <c r="AJ26" s="1045" t="n"/>
+      <c r="AE26" s="1291" t="inlineStr">
+        <is>
+          <t>ELDA LEAD LEADERS OFFICER</t>
+        </is>
+      </c>
+      <c r="AF26" s="1292" t="n"/>
+      <c r="AG26" s="1292" t="n"/>
+      <c r="AH26" s="1292" t="n"/>
+      <c r="AI26" s="1292" t="n"/>
+      <c r="AJ26" s="1292" t="n"/>
       <c r="AK26" s="1045" t="n"/>
       <c r="AN26" s="1149" t="n"/>
     </row>
@@ -8817,21 +8860,13 @@
       <c r="N33" s="1008" t="n"/>
       <c r="O33" s="1012" t="n"/>
       <c r="P33" s="1012" t="n"/>
-      <c r="Q33" s="1273" t="inlineStr">
-        <is>
-          <t>TTT WAI</t>
-        </is>
-      </c>
-      <c r="R33" s="1155" t="n"/>
-      <c r="S33" s="1156" t="n"/>
+      <c r="Q33" s="1287" t="n"/>
+      <c r="R33" s="1003" t="n"/>
+      <c r="S33" s="1003" t="n"/>
       <c r="T33" s="1008" t="n"/>
-      <c r="U33" s="1273" t="inlineStr">
-        <is>
-          <t>LEAD TEAMS</t>
-        </is>
-      </c>
-      <c r="V33" s="1155" t="n"/>
-      <c r="W33" s="1156" t="n"/>
+      <c r="U33" s="1287" t="n"/>
+      <c r="V33" s="1290" t="n"/>
+      <c r="W33" s="1290" t="n"/>
       <c r="X33" s="1008" t="n"/>
       <c r="Y33" s="1009" t="n"/>
       <c r="Z33" s="1009" t="n"/>
@@ -8868,18 +8903,14 @@
       <c r="V34" s="1012" t="n"/>
       <c r="W34" s="1012" t="n"/>
       <c r="X34" s="1008" t="n"/>
-      <c r="Y34" s="1274" t="inlineStr">
-        <is>
-          <t>LEAD SYS OFFICER</t>
-        </is>
-      </c>
-      <c r="Z34" s="1155" t="n"/>
-      <c r="AA34" s="1155" t="n"/>
-      <c r="AB34" s="1155" t="n"/>
-      <c r="AC34" s="1155" t="n"/>
-      <c r="AD34" s="1155" t="n"/>
-      <c r="AE34" s="1155" t="n"/>
-      <c r="AF34" s="1156" t="n"/>
+      <c r="Y34" s="1287" t="n"/>
+      <c r="Z34" s="1003" t="n"/>
+      <c r="AA34" s="1003" t="n"/>
+      <c r="AB34" s="1003" t="n"/>
+      <c r="AC34" s="1290" t="n"/>
+      <c r="AD34" s="1290" t="n"/>
+      <c r="AE34" s="1003" t="n"/>
+      <c r="AF34" s="1003" t="n"/>
       <c r="AG34" s="1022" t="n"/>
       <c r="AH34" s="1022" t="n"/>
       <c r="AI34" s="1012" t="n"/>
@@ -9020,13 +9051,21 @@
       <c r="N38" s="1013" t="n"/>
       <c r="O38" s="1012" t="n"/>
       <c r="P38" s="1015" t="n"/>
-      <c r="Q38" s="1064" t="n"/>
-      <c r="R38" s="1022" t="n"/>
-      <c r="S38" s="1022" t="n"/>
+      <c r="Q38" s="1245" t="inlineStr">
+        <is>
+          <t>LD TTT WAI</t>
+        </is>
+      </c>
+      <c r="R38" s="1293" t="n"/>
+      <c r="S38" s="1293" t="n"/>
       <c r="T38" s="1024" t="n"/>
-      <c r="U38" s="1022" t="n"/>
-      <c r="V38" s="1044" t="n"/>
-      <c r="W38" s="1044" t="n"/>
+      <c r="U38" s="1288" t="inlineStr">
+        <is>
+          <t>LD LEAD TEAMS</t>
+        </is>
+      </c>
+      <c r="V38" s="1289" t="n"/>
+      <c r="W38" s="1289" t="n"/>
       <c r="X38" s="1008" t="n"/>
       <c r="Y38" s="1008" t="n"/>
       <c r="Z38" s="1022" t="n"/>
@@ -9067,14 +9106,18 @@
       <c r="V39" s="1012" t="n"/>
       <c r="W39" s="1012" t="n"/>
       <c r="X39" s="1008" t="n"/>
-      <c r="Y39" s="1022" t="n"/>
-      <c r="Z39" s="1022" t="n"/>
-      <c r="AA39" s="1022" t="n"/>
-      <c r="AB39" s="1022" t="n"/>
-      <c r="AC39" s="1044" t="n"/>
-      <c r="AD39" s="1044" t="n"/>
-      <c r="AE39" s="1022" t="n"/>
-      <c r="AF39" s="1022" t="n"/>
+      <c r="Y39" s="1291" t="inlineStr">
+        <is>
+          <t>ELDA LEAD SYS OFFICER</t>
+        </is>
+      </c>
+      <c r="Z39" s="1292" t="n"/>
+      <c r="AA39" s="1292" t="n"/>
+      <c r="AB39" s="1292" t="n"/>
+      <c r="AC39" s="1292" t="n"/>
+      <c r="AD39" s="1292" t="n"/>
+      <c r="AE39" s="1292" t="n"/>
+      <c r="AF39" s="1292" t="n"/>
       <c r="AG39" s="1022" t="n"/>
       <c r="AH39" s="1022" t="n"/>
       <c r="AI39" s="1012" t="n"/>
@@ -9682,7 +9725,7 @@
       <c r="AD52" s="1012" t="n"/>
       <c r="AE52" s="1274" t="inlineStr">
         <is>
-          <t>LEAD LEADERS BMC</t>
+          <t>ELDA LEAD LEADERS BMC</t>
         </is>
       </c>
       <c r="AF52" s="1155" t="n"/>
@@ -10219,7 +10262,7 @@
       <c r="I64" s="1090" t="n"/>
       <c r="J64" s="1273" t="inlineStr">
         <is>
-          <t>LEAD LEADERS 27_03 BMC</t>
+          <t>LD LEAD LEADERS 27_03 BMC</t>
         </is>
       </c>
       <c r="K64" s="1155" t="n"/>
@@ -10237,7 +10280,7 @@
       <c r="W64" s="1091" t="n"/>
       <c r="X64" s="1273" t="inlineStr">
         <is>
-          <t>LEAD TEAMS BMC</t>
+          <t>LD LEAD TEAMS BMC</t>
         </is>
       </c>
       <c r="Y64" s="1155" t="n"/>
@@ -10274,7 +10317,7 @@
       <c r="P65" s="1012" t="n"/>
       <c r="Q65" s="1274" t="inlineStr">
         <is>
-          <t>LEAD TEAMS BMC</t>
+          <t>ELDA LEAD TEAMS BMC</t>
         </is>
       </c>
       <c r="R65" s="1155" t="n"/>
@@ -10292,7 +10335,7 @@
       <c r="AD65" s="1012" t="n"/>
       <c r="AE65" s="1274" t="inlineStr">
         <is>
-          <t>LEAD TEAMS LTN</t>
+          <t>ELDA LEAD TEAMS LTN</t>
         </is>
       </c>
       <c r="AF65" s="1155" t="n"/>
@@ -10825,7 +10868,7 @@
       <c r="C77" s="1149" t="n"/>
       <c r="D77" s="1273" t="inlineStr">
         <is>
-          <t>LEAD TEAMS LTN</t>
+          <t>LD LEAD TEAMS LTN</t>
         </is>
       </c>
       <c r="E77" s="1155" t="n"/>
@@ -10882,7 +10925,7 @@
       <c r="Q78" s="1008" t="n"/>
       <c r="R78" s="1274" t="inlineStr">
         <is>
-          <t>LEAD SYS</t>
+          <t>ELDA LEAD SYS</t>
         </is>
       </c>
       <c r="S78" s="1155" t="n"/>
@@ -12084,7 +12127,7 @@
       <c r="M104" s="1008" t="n"/>
       <c r="N104" s="1274" t="inlineStr">
         <is>
-          <t>LEAD SYS (ADV RACE)</t>
+          <t>ELDA LEAD SYS (ADV RACE)</t>
         </is>
       </c>
       <c r="O104" s="1155" t="n"/>
@@ -12105,7 +12148,7 @@
       <c r="AD104" s="1012" t="n"/>
       <c r="AE104" s="1274" t="inlineStr">
         <is>
-          <t>LEAD SYS (ALPINE TOUR)</t>
+          <t>ELDA LEAD SYS (ALPINE TOUR)</t>
         </is>
       </c>
       <c r="AF104" s="1155" t="n"/>
@@ -12116,7 +12159,7 @@
       <c r="AK104" s="1156" t="n"/>
       <c r="AL104" s="1274" t="inlineStr">
         <is>
-          <t>LEAD TEAMS</t>
+          <t>ELDA LEAD TEAMS</t>
         </is>
       </c>
       <c r="AM104" s="1156" t="n"/>
@@ -12676,7 +12719,7 @@
       <c r="I117" s="1044" t="n"/>
       <c r="J117" s="1273" t="inlineStr">
         <is>
-          <t>LEAD TEAMS BMC</t>
+          <t>LD LEAD TEAMS BMC</t>
         </is>
       </c>
       <c r="K117" s="1155" t="n"/>
@@ -12694,7 +12737,7 @@
       <c r="W117" s="1108" t="n"/>
       <c r="X117" s="1273" t="inlineStr">
         <is>
-          <t>LEAD TEAMS LTN</t>
+          <t>LD LEAD TEAMS LTN</t>
         </is>
       </c>
       <c r="Y117" s="1155" t="n"/>
@@ -12718,7 +12761,7 @@
       <c r="D118" s="1149" t="n"/>
       <c r="E118" s="1274" t="inlineStr">
         <is>
-          <t>LEAD TEAMS BMC</t>
+          <t>ELDA LEAD TEAMS BMC</t>
         </is>
       </c>
       <c r="F118" s="1155" t="n"/>
@@ -12734,7 +12777,7 @@
       <c r="P118" s="1044" t="n"/>
       <c r="Q118" s="1274" t="inlineStr">
         <is>
-          <t>LEAD TEAMS LTN</t>
+          <t>ELDA LEAD TEAMS LTN</t>
         </is>
       </c>
       <c r="R118" s="1155" t="n"/>
@@ -12751,7 +12794,7 @@
       <c r="AC118" s="1044" t="n"/>
       <c r="AD118" s="1274" t="inlineStr">
         <is>
-          <t>LEAD LEADERS</t>
+          <t>ELDA LEAD LEADERS</t>
         </is>
       </c>
       <c r="AE118" s="1155" t="n"/>
@@ -13289,7 +13332,7 @@
       <c r="I130" s="1091" t="n"/>
       <c r="J130" s="1273" t="inlineStr">
         <is>
-          <t>LEAD LEADERS</t>
+          <t>LD LEAD LEADERS</t>
         </is>
       </c>
       <c r="K130" s="1155" t="n"/>
@@ -13339,7 +13382,7 @@
       <c r="O131" s="1043" t="n"/>
       <c r="P131" s="1274" t="inlineStr">
         <is>
-          <t>LEAD LEADERS (OFFICERS)</t>
+          <t>ELDA LEAD LEADERS (OFFICERS)</t>
         </is>
       </c>
       <c r="Q131" s="1155" t="n"/>
@@ -13926,7 +13969,7 @@
       <c r="O144" s="1043" t="n"/>
       <c r="P144" s="1274" t="inlineStr">
         <is>
-          <t>LEAD INTEGRATED CAP</t>
+          <t>ELDA LEAD INTEGRATED CAP</t>
         </is>
       </c>
       <c r="Q144" s="1155" t="n"/>
@@ -15039,6 +15082,7 @@
     <mergeCell ref="AK105:AM105"/>
     <mergeCell ref="AH71:AN82"/>
     <mergeCell ref="L11:N11"/>
+    <mergeCell ref="J25:N25"/>
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="D77:G77"/>
     <mergeCell ref="B137:I148"/>
@@ -15046,7 +15090,6 @@
     <mergeCell ref="AJ45:AN56"/>
     <mergeCell ref="F87:Q87"/>
     <mergeCell ref="D79:AG79"/>
-    <mergeCell ref="Q33:S33"/>
     <mergeCell ref="J130:N130"/>
     <mergeCell ref="A59:A60"/>
     <mergeCell ref="B97:H109"/>
@@ -15058,12 +15101,12 @@
     <mergeCell ref="J145:P145"/>
     <mergeCell ref="AL104:AM104"/>
     <mergeCell ref="J151:N160"/>
-    <mergeCell ref="J24:N24"/>
     <mergeCell ref="A114:A116"/>
     <mergeCell ref="A46:A47"/>
     <mergeCell ref="A21:A24"/>
     <mergeCell ref="AM58:AN69"/>
     <mergeCell ref="AE52:AI52"/>
+    <mergeCell ref="U38:W38"/>
     <mergeCell ref="J120:AH120"/>
     <mergeCell ref="P107:AC107"/>
     <mergeCell ref="AE80:AG80"/>
@@ -15077,16 +15120,18 @@
     <mergeCell ref="B18:I30"/>
     <mergeCell ref="B150:D161"/>
     <mergeCell ref="A74:A76"/>
+    <mergeCell ref="X25:AB25"/>
     <mergeCell ref="D81:U81"/>
     <mergeCell ref="P131:U131"/>
     <mergeCell ref="J42:W42"/>
+    <mergeCell ref="G131:H131"/>
     <mergeCell ref="J147:AB147"/>
-    <mergeCell ref="G131:H131"/>
     <mergeCell ref="AN97:AN109"/>
     <mergeCell ref="V41:AB41"/>
     <mergeCell ref="AE13:AK13"/>
     <mergeCell ref="X11:AB11"/>
     <mergeCell ref="A100:A102"/>
+    <mergeCell ref="Q26:V26"/>
     <mergeCell ref="AE104:AK104"/>
     <mergeCell ref="Q114:AH114"/>
     <mergeCell ref="Q65:V65"/>
@@ -15094,8 +15139,6 @@
     <mergeCell ref="F93:N93"/>
     <mergeCell ref="AE65:AJ65"/>
     <mergeCell ref="A127:A129"/>
-    <mergeCell ref="X24:AB24"/>
-    <mergeCell ref="Y34:AF34"/>
     <mergeCell ref="A87:A89"/>
     <mergeCell ref="V81:AB81"/>
     <mergeCell ref="J28:AK28"/>
@@ -15117,6 +15160,7 @@
     <mergeCell ref="AE12:AJ12"/>
     <mergeCell ref="AE55:AI55"/>
     <mergeCell ref="B111:D122"/>
+    <mergeCell ref="Q38:S38"/>
     <mergeCell ref="O7:AK7"/>
     <mergeCell ref="J36:U36"/>
     <mergeCell ref="AL4:AN16"/>
@@ -15124,10 +15168,10 @@
     <mergeCell ref="X119:AH119"/>
     <mergeCell ref="AE133:AK133"/>
     <mergeCell ref="A140:A142"/>
+    <mergeCell ref="Y39:AF39"/>
     <mergeCell ref="F55:G55"/>
     <mergeCell ref="A35:A37"/>
     <mergeCell ref="M23:AB23"/>
-    <mergeCell ref="U33:W33"/>
     <mergeCell ref="AC92:AJ92"/>
     <mergeCell ref="A108:A109"/>
     <mergeCell ref="AJ150:AN161"/>
@@ -15141,14 +15185,13 @@
     <mergeCell ref="AC145:AI145"/>
     <mergeCell ref="A72:A73"/>
     <mergeCell ref="AE121:AH121"/>
+    <mergeCell ref="AE26:AJ26"/>
     <mergeCell ref="X117:AB117"/>
     <mergeCell ref="S100:AD100"/>
-    <mergeCell ref="Q25:V25"/>
     <mergeCell ref="AC147:AI147"/>
     <mergeCell ref="Q67:AL67"/>
     <mergeCell ref="X40:AI40"/>
     <mergeCell ref="O146:U146"/>
-    <mergeCell ref="AE25:AJ25"/>
     <mergeCell ref="O93:U93"/>
     <mergeCell ref="AL18:AN30"/>
     <mergeCell ref="X74:AG74"/>

</xml_diff>

<commit_message>
March schedule edits: remove LD TTT WAI, shift LD Lead Teams
LD TTT WAI (8-10 Mar) is removed and LD Lead Teams moves from
12-14 Mar to 19-21 Mar. Vacated cells return to plain grid styling.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLo1WfwUDkbwfJEF3ZNVbB
</commit_message>
<xml_diff>
--- a/output/acs-activity-calendar-2027.xlsx
+++ b/output/acs-activity-calendar-2027.xlsx
@@ -2598,7 +2598,7 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1294">
+  <cellXfs count="1295">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -6515,6 +6515,10 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="53" borderId="146" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="103" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8455,10 +8459,10 @@
           <t>LD LEAD TEAMS LMC</t>
         </is>
       </c>
-      <c r="K25" s="1289" t="n"/>
-      <c r="L25" s="1289" t="n"/>
-      <c r="M25" s="1289" t="n"/>
-      <c r="N25" s="1289" t="n"/>
+      <c r="K25" s="844" t="n"/>
+      <c r="L25" s="844" t="n"/>
+      <c r="M25" s="844" t="n"/>
+      <c r="N25" s="844" t="n"/>
       <c r="O25" s="1012" t="n"/>
       <c r="P25" s="1012" t="n"/>
       <c r="Q25" s="1287" t="n"/>
@@ -8473,10 +8477,10 @@
           <t>LD LEAD LEADERS BMC</t>
         </is>
       </c>
-      <c r="Y25" s="1289" t="n"/>
-      <c r="Z25" s="1289" t="n"/>
-      <c r="AA25" s="1289" t="n"/>
-      <c r="AB25" s="1289" t="n"/>
+      <c r="Y25" s="844" t="n"/>
+      <c r="Z25" s="844" t="n"/>
+      <c r="AA25" s="844" t="n"/>
+      <c r="AB25" s="844" t="n"/>
       <c r="AC25" s="1012" t="n"/>
       <c r="AD25" s="1012" t="n"/>
       <c r="AE25" s="1287" t="n"/>
@@ -8507,11 +8511,11 @@
           <t>ELDA LEAD LEADERS BMC</t>
         </is>
       </c>
-      <c r="R26" s="1292" t="n"/>
-      <c r="S26" s="1292" t="n"/>
-      <c r="T26" s="1292" t="n"/>
-      <c r="U26" s="1292" t="n"/>
-      <c r="V26" s="1292" t="n"/>
+      <c r="R26" s="844" t="n"/>
+      <c r="S26" s="844" t="n"/>
+      <c r="T26" s="844" t="n"/>
+      <c r="U26" s="844" t="n"/>
+      <c r="V26" s="844" t="n"/>
       <c r="W26" s="1012" t="n"/>
       <c r="X26" s="1024" t="n"/>
       <c r="Y26" s="1024" t="n"/>
@@ -8525,11 +8529,11 @@
           <t>ELDA LEAD LEADERS OFFICER</t>
         </is>
       </c>
-      <c r="AF26" s="1292" t="n"/>
-      <c r="AG26" s="1292" t="n"/>
-      <c r="AH26" s="1292" t="n"/>
-      <c r="AI26" s="1292" t="n"/>
-      <c r="AJ26" s="1292" t="n"/>
+      <c r="AF26" s="844" t="n"/>
+      <c r="AG26" s="844" t="n"/>
+      <c r="AH26" s="844" t="n"/>
+      <c r="AI26" s="844" t="n"/>
+      <c r="AJ26" s="844" t="n"/>
       <c r="AK26" s="1045" t="n"/>
       <c r="AN26" s="1149" t="n"/>
     </row>
@@ -9051,28 +9055,24 @@
       <c r="N38" s="1013" t="n"/>
       <c r="O38" s="1012" t="n"/>
       <c r="P38" s="1015" t="n"/>
-      <c r="Q38" s="1245" t="inlineStr">
-        <is>
-          <t>LD TTT WAI</t>
-        </is>
-      </c>
-      <c r="R38" s="1293" t="n"/>
-      <c r="S38" s="1293" t="n"/>
+      <c r="Q38" s="1287" t="n"/>
+      <c r="R38" s="1003" t="n"/>
+      <c r="S38" s="1003" t="n"/>
       <c r="T38" s="1024" t="n"/>
-      <c r="U38" s="1288" t="inlineStr">
-        <is>
-          <t>LD LEAD TEAMS</t>
-        </is>
-      </c>
-      <c r="V38" s="1289" t="n"/>
-      <c r="W38" s="1289" t="n"/>
+      <c r="U38" s="1294" t="n"/>
+      <c r="V38" s="1290" t="n"/>
+      <c r="W38" s="1290" t="n"/>
       <c r="X38" s="1008" t="n"/>
       <c r="Y38" s="1008" t="n"/>
       <c r="Z38" s="1022" t="n"/>
       <c r="AA38" s="1022" t="n"/>
-      <c r="AB38" s="1022" t="n"/>
-      <c r="AC38" s="1044" t="n"/>
-      <c r="AD38" s="1044" t="n"/>
+      <c r="AB38" s="1288" t="inlineStr">
+        <is>
+          <t>LD LEAD TEAMS</t>
+        </is>
+      </c>
+      <c r="AC38" s="1289" t="n"/>
+      <c r="AD38" s="1289" t="n"/>
       <c r="AE38" s="1022" t="n"/>
       <c r="AF38" s="1022" t="n"/>
       <c r="AG38" s="1022" t="n"/>
@@ -9111,13 +9111,13 @@
           <t>ELDA LEAD SYS OFFICER</t>
         </is>
       </c>
-      <c r="Z39" s="1292" t="n"/>
-      <c r="AA39" s="1292" t="n"/>
-      <c r="AB39" s="1292" t="n"/>
-      <c r="AC39" s="1292" t="n"/>
-      <c r="AD39" s="1292" t="n"/>
-      <c r="AE39" s="1292" t="n"/>
-      <c r="AF39" s="1292" t="n"/>
+      <c r="Z39" s="844" t="n"/>
+      <c r="AA39" s="844" t="n"/>
+      <c r="AB39" s="844" t="n"/>
+      <c r="AC39" s="844" t="n"/>
+      <c r="AD39" s="844" t="n"/>
+      <c r="AE39" s="844" t="n"/>
+      <c r="AF39" s="844" t="n"/>
       <c r="AG39" s="1022" t="n"/>
       <c r="AH39" s="1022" t="n"/>
       <c r="AI39" s="1012" t="n"/>
@@ -15057,7 +15057,7 @@
       <c r="AN164" s="1225" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="141">
+  <mergeCells count="140">
     <mergeCell ref="AK84:AN95"/>
     <mergeCell ref="Q118:V118"/>
     <mergeCell ref="J64:N64"/>
@@ -15106,7 +15106,6 @@
     <mergeCell ref="A21:A24"/>
     <mergeCell ref="AM58:AN69"/>
     <mergeCell ref="AE52:AI52"/>
-    <mergeCell ref="U38:W38"/>
     <mergeCell ref="J120:AH120"/>
     <mergeCell ref="P107:AC107"/>
     <mergeCell ref="AE80:AG80"/>
@@ -15124,8 +15123,8 @@
     <mergeCell ref="D81:U81"/>
     <mergeCell ref="P131:U131"/>
     <mergeCell ref="J42:W42"/>
+    <mergeCell ref="J147:AB147"/>
     <mergeCell ref="G131:H131"/>
-    <mergeCell ref="J147:AB147"/>
     <mergeCell ref="AN97:AN109"/>
     <mergeCell ref="V41:AB41"/>
     <mergeCell ref="AE13:AK13"/>
@@ -15134,6 +15133,7 @@
     <mergeCell ref="Q26:V26"/>
     <mergeCell ref="AE104:AK104"/>
     <mergeCell ref="Q114:AH114"/>
+    <mergeCell ref="AB38:AD38"/>
     <mergeCell ref="Q65:V65"/>
     <mergeCell ref="J41:U41"/>
     <mergeCell ref="F93:N93"/>
@@ -15160,7 +15160,6 @@
     <mergeCell ref="AE12:AJ12"/>
     <mergeCell ref="AE55:AI55"/>
     <mergeCell ref="B111:D122"/>
-    <mergeCell ref="Q38:S38"/>
     <mergeCell ref="O7:AK7"/>
     <mergeCell ref="J36:U36"/>
     <mergeCell ref="AL4:AN16"/>

</xml_diff>

<commit_message>
ELDA Lead Leaders across the month boundary; cover page trimmed to v1.0
Calendar: the April ELDA course is renamed to ELDA Lead Leaders and now
runs 26 April to 1 May, with the one-day continuation carried onto May's
ELDA row.

Proposal cover: the descriptive sentence under the red rule and the
tagline qualifier are removed, leaving the two tagline lines. Version
moves to Draft v1.0.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLo1WfwUDkbwfJEF3ZNVbB
</commit_message>
<xml_diff>
--- a/output/acs-activity-calendar-2027.xlsx
+++ b/output/acs-activity-calendar-2027.xlsx
@@ -828,7 +828,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="155">
+  <borders count="156">
     <border>
       <left/>
       <right/>
@@ -2578,6 +2578,10 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2598,7 +2602,7 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1295">
+  <cellXfs count="1297">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -6516,6 +6520,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="53" borderId="146" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="103" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="53" borderId="155" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="54" borderId="155" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -8454,7 +8466,7 @@
         </is>
       </c>
       <c r="I25" s="1149" t="n"/>
-      <c r="J25" s="1288" t="inlineStr">
+      <c r="J25" s="1295" t="inlineStr">
         <is>
           <t>LD LEAD TEAMS LMC</t>
         </is>
@@ -8472,7 +8484,7 @@
       <c r="U25" s="1003" t="n"/>
       <c r="V25" s="1290" t="n"/>
       <c r="W25" s="1012" t="n"/>
-      <c r="X25" s="1288" t="inlineStr">
+      <c r="X25" s="1295" t="inlineStr">
         <is>
           <t>LD LEAD LEADERS BMC</t>
         </is>
@@ -8506,7 +8518,7 @@
       <c r="N26" s="1008" t="n"/>
       <c r="O26" s="1012" t="n"/>
       <c r="P26" s="1012" t="n"/>
-      <c r="Q26" s="1291" t="inlineStr">
+      <c r="Q26" s="1296" t="inlineStr">
         <is>
           <t>ELDA LEAD LEADERS BMC</t>
         </is>
@@ -8524,7 +8536,7 @@
       <c r="AB26" s="1024" t="n"/>
       <c r="AC26" s="1043" t="n"/>
       <c r="AD26" s="1012" t="n"/>
-      <c r="AE26" s="1291" t="inlineStr">
+      <c r="AE26" s="1296" t="inlineStr">
         <is>
           <t>ELDA LEAD LEADERS OFFICER</t>
         </is>
@@ -9066,13 +9078,13 @@
       <c r="Y38" s="1008" t="n"/>
       <c r="Z38" s="1022" t="n"/>
       <c r="AA38" s="1022" t="n"/>
-      <c r="AB38" s="1288" t="inlineStr">
+      <c r="AB38" s="1295" t="inlineStr">
         <is>
           <t>LD LEAD TEAMS</t>
         </is>
       </c>
-      <c r="AC38" s="1289" t="n"/>
-      <c r="AD38" s="1289" t="n"/>
+      <c r="AC38" s="844" t="n"/>
+      <c r="AD38" s="844" t="n"/>
       <c r="AE38" s="1022" t="n"/>
       <c r="AF38" s="1022" t="n"/>
       <c r="AG38" s="1022" t="n"/>
@@ -9106,7 +9118,7 @@
       <c r="V39" s="1012" t="n"/>
       <c r="W39" s="1012" t="n"/>
       <c r="X39" s="1008" t="n"/>
-      <c r="Y39" s="1291" t="inlineStr">
+      <c r="Y39" s="1296" t="inlineStr">
         <is>
           <t>ELDA LEAD SYS OFFICER</t>
         </is>
@@ -9725,7 +9737,7 @@
       <c r="AD52" s="1012" t="n"/>
       <c r="AE52" s="1274" t="inlineStr">
         <is>
-          <t>ELDA LEAD LEADERS BMC</t>
+          <t>ELDA LEAD LEADERS</t>
         </is>
       </c>
       <c r="AF52" s="1155" t="n"/>
@@ -10306,7 +10318,11 @@
         </is>
       </c>
       <c r="G65" s="1149" t="n"/>
-      <c r="H65" s="1012" t="n"/>
+      <c r="H65" s="1291" t="inlineStr">
+        <is>
+          <t>ELDA</t>
+        </is>
+      </c>
       <c r="I65" s="1012" t="n"/>
       <c r="J65" s="1008" t="n"/>
       <c r="K65" s="1008" t="n"/>

</xml_diff>